<commit_message>
feat(examples): add interrupt and raw load/store programs
Normalize the load/store image filename and update the RC instruction layout in the ISA workbook.
</commit_message>
<xml_diff>
--- a/document/isa.xlsx
+++ b/document/isa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Project\Sipeed\FPGA\Tang_Primer\CPU\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C151930-06A6-4E1E-B01D-E2A18A205CB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A34BE91D-A578-41C5-A088-848775C3768F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="62">
   <si>
     <t>opcode</t>
   </si>
@@ -241,6 +241,10 @@
   </si>
   <si>
     <t>Jump And Link: 程序无条件跳转到IMM执行，并将函数返回地址保存到 rd 中</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>XXXXXXXXXXX</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1540,18 +1544,14 @@
       <c r="E33" s="7"/>
       <c r="F33" s="7"/>
       <c r="G33" s="6" t="s">
-        <v>4</v>
+        <v>61</v>
       </c>
       <c r="H33" s="6"/>
       <c r="I33" s="6"/>
-      <c r="J33" s="6" t="s">
-        <v>4</v>
-      </c>
+      <c r="J33" s="6"/>
       <c r="K33" s="6"/>
       <c r="L33" s="6"/>
-      <c r="M33" s="6" t="s">
-        <v>5</v>
-      </c>
+      <c r="M33" s="6"/>
       <c r="N33" s="6"/>
       <c r="O33" s="6"/>
       <c r="P33" s="6"/>
@@ -1562,16 +1562,78 @@
       <c r="T33" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="105">
-    <mergeCell ref="J16:L16"/>
-    <mergeCell ref="J17:L17"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="G23:I23"/>
-    <mergeCell ref="J20:L20"/>
-    <mergeCell ref="J21:L21"/>
-    <mergeCell ref="J22:L22"/>
-    <mergeCell ref="J23:L23"/>
-    <mergeCell ref="J25:L25"/>
+  <mergeCells count="103">
+    <mergeCell ref="M18:Q18"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="J27:L27"/>
+    <mergeCell ref="M27:Q27"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="M20:Q20"/>
+    <mergeCell ref="M21:Q21"/>
+    <mergeCell ref="M22:Q22"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="G32:I32"/>
+    <mergeCell ref="J32:Q32"/>
+    <mergeCell ref="B23:F23"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="G30:I30"/>
+    <mergeCell ref="M23:Q23"/>
+    <mergeCell ref="M25:Q25"/>
+    <mergeCell ref="M28:Q28"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="G28:I28"/>
+    <mergeCell ref="J26:L26"/>
+    <mergeCell ref="M26:Q26"/>
+    <mergeCell ref="J28:L28"/>
+    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="J30:Q30"/>
+    <mergeCell ref="J31:Q31"/>
+    <mergeCell ref="G33:Q33"/>
+    <mergeCell ref="M19:Q19"/>
+    <mergeCell ref="M10:Q10"/>
+    <mergeCell ref="M11:Q11"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="J12:L12"/>
+    <mergeCell ref="M12:Q12"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="M16:Q16"/>
+    <mergeCell ref="M17:Q17"/>
+    <mergeCell ref="M6:Q6"/>
+    <mergeCell ref="M7:Q7"/>
+    <mergeCell ref="M8:Q8"/>
+    <mergeCell ref="M9:Q9"/>
+    <mergeCell ref="J9:L9"/>
+    <mergeCell ref="J10:L10"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="G2:I2"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="M2:Q2"/>
+    <mergeCell ref="J3:L3"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="J8:L8"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="M3:Q3"/>
+    <mergeCell ref="M4:Q4"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="M5:Q5"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="B22:F22"/>
     <mergeCell ref="B25:F25"/>
@@ -1592,82 +1654,18 @@
     <mergeCell ref="G22:I22"/>
     <mergeCell ref="G25:I25"/>
     <mergeCell ref="G26:I26"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="G2:I2"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="M2:Q2"/>
-    <mergeCell ref="J3:L3"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="J7:L7"/>
-    <mergeCell ref="J8:L8"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="M19:Q19"/>
-    <mergeCell ref="M10:Q10"/>
-    <mergeCell ref="M11:Q11"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="J12:L12"/>
-    <mergeCell ref="M12:Q12"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="M16:Q16"/>
-    <mergeCell ref="M17:Q17"/>
-    <mergeCell ref="M3:Q3"/>
-    <mergeCell ref="M4:Q4"/>
-    <mergeCell ref="M6:Q6"/>
-    <mergeCell ref="M7:Q7"/>
-    <mergeCell ref="M8:Q8"/>
-    <mergeCell ref="M9:Q9"/>
-    <mergeCell ref="J9:L9"/>
-    <mergeCell ref="J10:L10"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="B33:F33"/>
-    <mergeCell ref="G32:I32"/>
-    <mergeCell ref="J32:Q32"/>
-    <mergeCell ref="B23:F23"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="G33:I33"/>
-    <mergeCell ref="J33:L33"/>
-    <mergeCell ref="M33:Q33"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="G30:I30"/>
-    <mergeCell ref="M23:Q23"/>
-    <mergeCell ref="M25:Q25"/>
-    <mergeCell ref="M28:Q28"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="G28:I28"/>
-    <mergeCell ref="J26:L26"/>
-    <mergeCell ref="M26:Q26"/>
-    <mergeCell ref="J28:L28"/>
-    <mergeCell ref="G31:I31"/>
-    <mergeCell ref="J30:Q30"/>
-    <mergeCell ref="J31:Q31"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="B8:F8"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
     <mergeCell ref="B12:F12"/>
-    <mergeCell ref="G5:I5"/>
-    <mergeCell ref="J5:L5"/>
-    <mergeCell ref="M5:Q5"/>
     <mergeCell ref="G18:I18"/>
+    <mergeCell ref="J16:L16"/>
+    <mergeCell ref="J17:L17"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="G23:I23"/>
+    <mergeCell ref="J20:L20"/>
+    <mergeCell ref="J21:L21"/>
+    <mergeCell ref="J22:L22"/>
+    <mergeCell ref="J23:L23"/>
+    <mergeCell ref="J25:L25"/>
     <mergeCell ref="J18:L18"/>
-    <mergeCell ref="M18:Q18"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="J27:L27"/>
-    <mergeCell ref="M27:Q27"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="M20:Q20"/>
-    <mergeCell ref="M21:Q21"/>
-    <mergeCell ref="M22:Q22"/>
-    <mergeCell ref="B19:F19"/>
-    <mergeCell ref="B20:F20"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
chore: clear GUI test scripts and refresh project documentation
Clear GUI_v1/test1.py and GUI_v2/test2.py, reindent the README header, and refresh the ISA workbook.
</commit_message>
<xml_diff>
--- a/document/isa.xlsx
+++ b/document/isa.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Project\Sipeed\FPGA\Tang_Primer\CPU\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A34BE91D-A578-41C5-A088-848775C3768F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57F8018F-ED8D-485D-A678-1CE0A34DBFAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11796" yWindow="2916" windowWidth="11244" windowHeight="9444" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1563,17 +1563,63 @@
     </row>
   </sheetData>
   <mergeCells count="103">
-    <mergeCell ref="M18:Q18"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="J27:L27"/>
-    <mergeCell ref="M27:Q27"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="M20:Q20"/>
-    <mergeCell ref="M21:Q21"/>
-    <mergeCell ref="M22:Q22"/>
-    <mergeCell ref="B19:F19"/>
-    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="G22:I22"/>
+    <mergeCell ref="G25:I25"/>
+    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="G18:I18"/>
+    <mergeCell ref="J16:L16"/>
+    <mergeCell ref="J17:L17"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="G23:I23"/>
+    <mergeCell ref="J20:L20"/>
+    <mergeCell ref="J21:L21"/>
+    <mergeCell ref="J22:L22"/>
+    <mergeCell ref="J23:L23"/>
+    <mergeCell ref="J25:L25"/>
+    <mergeCell ref="J18:L18"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="G2:I2"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="M2:Q2"/>
+    <mergeCell ref="J3:L3"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="J8:L8"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="M3:Q3"/>
+    <mergeCell ref="M4:Q4"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="M5:Q5"/>
+    <mergeCell ref="G3:I3"/>
+    <mergeCell ref="G4:I4"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="M16:Q16"/>
+    <mergeCell ref="M17:Q17"/>
+    <mergeCell ref="M6:Q6"/>
+    <mergeCell ref="M7:Q7"/>
+    <mergeCell ref="M8:Q8"/>
+    <mergeCell ref="M9:Q9"/>
+    <mergeCell ref="J9:L9"/>
+    <mergeCell ref="J10:L10"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="G17:I17"/>
     <mergeCell ref="B33:F33"/>
     <mergeCell ref="G32:I32"/>
     <mergeCell ref="J32:Q32"/>
@@ -1594,6 +1640,19 @@
     <mergeCell ref="J30:Q30"/>
     <mergeCell ref="J31:Q31"/>
     <mergeCell ref="G33:Q33"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="M18:Q18"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="J27:L27"/>
+    <mergeCell ref="M27:Q27"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="M20:Q20"/>
+    <mergeCell ref="M21:Q21"/>
+    <mergeCell ref="M22:Q22"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="B20:F20"/>
     <mergeCell ref="M19:Q19"/>
     <mergeCell ref="M10:Q10"/>
     <mergeCell ref="M11:Q11"/>
@@ -1601,71 +1660,12 @@
     <mergeCell ref="J12:L12"/>
     <mergeCell ref="M12:Q12"/>
     <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="M16:Q16"/>
-    <mergeCell ref="M17:Q17"/>
-    <mergeCell ref="M6:Q6"/>
-    <mergeCell ref="M7:Q7"/>
-    <mergeCell ref="M8:Q8"/>
-    <mergeCell ref="M9:Q9"/>
-    <mergeCell ref="J9:L9"/>
-    <mergeCell ref="J10:L10"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B17:F17"/>
     <mergeCell ref="B18:F18"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="B8:F8"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="G2:I2"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="M2:Q2"/>
-    <mergeCell ref="J3:L3"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="J7:L7"/>
-    <mergeCell ref="J8:L8"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="M3:Q3"/>
-    <mergeCell ref="M4:Q4"/>
-    <mergeCell ref="G5:I5"/>
-    <mergeCell ref="J5:L5"/>
-    <mergeCell ref="M5:Q5"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="B22:F22"/>
-    <mergeCell ref="B25:F25"/>
-    <mergeCell ref="B26:F26"/>
-    <mergeCell ref="G3:I3"/>
-    <mergeCell ref="G4:I4"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="G8:I8"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="G17:I17"/>
     <mergeCell ref="G19:I19"/>
     <mergeCell ref="G20:I20"/>
     <mergeCell ref="G21:I21"/>
-    <mergeCell ref="G22:I22"/>
-    <mergeCell ref="G25:I25"/>
-    <mergeCell ref="G26:I26"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="G18:I18"/>
-    <mergeCell ref="J16:L16"/>
-    <mergeCell ref="J17:L17"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="G23:I23"/>
-    <mergeCell ref="J20:L20"/>
-    <mergeCell ref="J21:L21"/>
-    <mergeCell ref="J22:L22"/>
-    <mergeCell ref="J23:L23"/>
-    <mergeCell ref="J25:L25"/>
-    <mergeCell ref="J18:L18"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>